<commit_message>
Update on UEFA Stats 2018
</commit_message>
<xml_diff>
--- a/Data/UEFA Stats 2018_with_IDs.xlsx
+++ b/Data/UEFA Stats 2018_with_IDs.xlsx
@@ -2919,7 +2919,7 @@
         <v>21.5</v>
       </c>
       <c r="J11">
-        <v>15956</v>
+        <v>79422</v>
       </c>
     </row>
     <row r="12" spans="1:10">
@@ -3143,7 +3143,7 @@
         <v>31.5</v>
       </c>
       <c r="J18">
-        <v>288230</v>
+        <v>200512</v>
       </c>
     </row>
     <row r="19" spans="1:10">
@@ -4359,7 +4359,7 @@
         <v>32.5</v>
       </c>
       <c r="J56">
-        <v>40433</v>
+        <v>341429</v>
       </c>
     </row>
     <row r="57" spans="1:10">
@@ -4743,7 +4743,7 @@
         <v>28.4</v>
       </c>
       <c r="J68">
-        <v>811779</v>
+        <v>93795</v>
       </c>
     </row>
     <row r="69" spans="1:10">
@@ -5863,7 +5863,7 @@
         <v>32</v>
       </c>
       <c r="J103">
-        <v>181767</v>
+        <v>227081</v>
       </c>
     </row>
     <row r="104" spans="1:10">
@@ -6055,7 +6055,7 @@
         <v>30.2</v>
       </c>
       <c r="J109">
-        <v>3924</v>
+        <v>175722</v>
       </c>
     </row>
     <row r="110" spans="1:10">
@@ -6215,7 +6215,7 @@
         <v>30.1</v>
       </c>
       <c r="J114">
-        <v>7476</v>
+        <v>112515</v>
       </c>
     </row>
     <row r="115" spans="1:10">
@@ -6567,7 +6567,7 @@
         <v>30.4</v>
       </c>
       <c r="J125">
-        <v>741238</v>
+        <v>16101</v>
       </c>
     </row>
     <row r="126" spans="1:10">
@@ -6855,7 +6855,7 @@
         <v>28</v>
       </c>
       <c r="J134">
-        <v>3394</v>
+        <v>48859</v>
       </c>
     </row>
     <row r="135" spans="1:10">
@@ -7623,7 +7623,7 @@
         <v>23.6</v>
       </c>
       <c r="J158">
-        <v>503733</v>
+        <v>12589</v>
       </c>
     </row>
     <row r="159" spans="1:10">
@@ -7719,7 +7719,7 @@
         <v>21.2</v>
       </c>
       <c r="J161">
-        <v>28021</v>
+        <v>47015</v>
       </c>
     </row>
     <row r="162" spans="1:10">
@@ -7879,7 +7879,7 @@
         <v>28.5</v>
       </c>
       <c r="J166">
-        <v>15646</v>
+        <v>89297</v>
       </c>
     </row>
     <row r="167" spans="1:10">
@@ -8039,7 +8039,7 @@
         <v>30.5</v>
       </c>
       <c r="J171">
-        <v>145707</v>
+        <v>141050</v>
       </c>
     </row>
     <row r="172" spans="1:10">
@@ -8199,7 +8199,7 @@
         <v>27.7</v>
       </c>
       <c r="J176">
-        <v>99343</v>
+        <v>122043</v>
       </c>
     </row>
     <row r="177" spans="1:10">
@@ -8647,7 +8647,7 @@
         <v>29.4</v>
       </c>
       <c r="J190">
-        <v>955070</v>
+        <v>111038</v>
       </c>
     </row>
     <row r="191" spans="1:10">
@@ -8743,7 +8743,7 @@
         <v>32.6</v>
       </c>
       <c r="J193">
-        <v>129473</v>
+        <v>33947</v>
       </c>
     </row>
     <row r="194" spans="1:10">
@@ -8903,7 +8903,7 @@
         <v>29.1</v>
       </c>
       <c r="J198">
-        <v>532</v>
+        <v>105899</v>
       </c>
     </row>
     <row r="199" spans="1:10">
@@ -8999,7 +8999,7 @@
         <v>27.7</v>
       </c>
       <c r="J201">
-        <v>221316</v>
+        <v>76163</v>
       </c>
     </row>
     <row r="202" spans="1:10">
@@ -9447,7 +9447,7 @@
         <v>27.6</v>
       </c>
       <c r="J215">
-        <v>607224</v>
+        <v>113358</v>
       </c>
     </row>
     <row r="216" spans="1:10">
@@ -10119,7 +10119,7 @@
         <v>28.7</v>
       </c>
       <c r="J236">
-        <v>424204</v>
+        <v>192765</v>
       </c>
     </row>
     <row r="237" spans="1:10">
@@ -10567,7 +10567,7 @@
         <v>20.2</v>
       </c>
       <c r="J250">
-        <v>137457</v>
+        <v>249994</v>
       </c>
     </row>
     <row r="251" spans="1:10">
@@ -11047,7 +11047,7 @@
         <v>29.7</v>
       </c>
       <c r="J265">
-        <v>534033</v>
+        <v>207929</v>
       </c>
     </row>
     <row r="266" spans="1:10">
@@ -12199,7 +12199,7 @@
         <v>28.4</v>
       </c>
       <c r="J301">
-        <v>8056</v>
+        <v>31552</v>
       </c>
     </row>
     <row r="302" spans="1:10">
@@ -12391,7 +12391,7 @@
         <v>29.9</v>
       </c>
       <c r="J307">
-        <v>48280</v>
+        <v>256178</v>
       </c>
     </row>
     <row r="308" spans="1:10">
@@ -12551,7 +12551,7 @@
         <v>27</v>
       </c>
       <c r="J312">
-        <v>565424</v>
+        <v>182618</v>
       </c>
     </row>
     <row r="313" spans="1:10">
@@ -12775,7 +12775,7 @@
         <v>29.1</v>
       </c>
       <c r="J319">
-        <v>3625</v>
+        <v>122946</v>
       </c>
     </row>
     <row r="320" spans="1:10">
@@ -13479,7 +13479,7 @@
         <v>31.8</v>
       </c>
       <c r="J341">
-        <v>6119</v>
+        <v>46001</v>
       </c>
     </row>
     <row r="342" spans="1:10">
@@ -13767,7 +13767,7 @@
         <v>29</v>
       </c>
       <c r="J350">
-        <v>116743</v>
+        <v>277137</v>
       </c>
     </row>
     <row r="351" spans="1:10">
@@ -13799,7 +13799,7 @@
         <v>28.1</v>
       </c>
       <c r="J351">
-        <v>288230</v>
+        <v>19368</v>
       </c>
     </row>
     <row r="352" spans="1:10">
@@ -15495,7 +15495,7 @@
         <v>30.1</v>
       </c>
       <c r="J404">
-        <v>13091</v>
+        <v>216181</v>
       </c>
     </row>
     <row r="405" spans="1:10">
@@ -15783,7 +15783,7 @@
         <v>22.4</v>
       </c>
       <c r="J413">
-        <v>223</v>
+        <v>127202</v>
       </c>
     </row>
     <row r="414" spans="1:10">
@@ -15975,7 +15975,7 @@
         <v>29.5</v>
       </c>
       <c r="J419">
-        <v>266302</v>
+        <v>107010</v>
       </c>
     </row>
     <row r="420" spans="1:10">
@@ -16071,7 +16071,7 @@
         <v>28</v>
       </c>
       <c r="J422">
-        <v>288230</v>
+        <v>229004</v>
       </c>
     </row>
     <row r="423" spans="1:10">
@@ -16199,7 +16199,7 @@
         <v>28.8</v>
       </c>
       <c r="J426">
-        <v>375382</v>
+        <v>83466</v>
       </c>
     </row>
     <row r="427" spans="1:10">
@@ -16935,7 +16935,7 @@
         <v>28.9</v>
       </c>
       <c r="J449">
-        <v>7717</v>
+        <v>131090</v>
       </c>
     </row>
     <row r="450" spans="1:10">
@@ -16999,7 +16999,7 @@
         <v>28.4</v>
       </c>
       <c r="J451">
-        <v>250426</v>
+        <v>130765</v>
       </c>
     </row>
     <row r="452" spans="1:10">
@@ -17031,7 +17031,7 @@
         <v>28.4</v>
       </c>
       <c r="J452">
-        <v>234803</v>
+        <v>225452</v>
       </c>
     </row>
     <row r="453" spans="1:10">
@@ -17063,7 +17063,7 @@
         <v>31.5</v>
       </c>
       <c r="J453">
-        <v>346289</v>
+        <v>453594</v>
       </c>
     </row>
     <row r="454" spans="1:10">
@@ -17159,7 +17159,7 @@
         <v>29.1</v>
       </c>
       <c r="J456">
-        <v>282411</v>
+        <v>35564</v>
       </c>
     </row>
     <row r="457" spans="1:10">
@@ -18471,7 +18471,7 @@
         <v>23.6</v>
       </c>
       <c r="J497">
-        <v>3979</v>
+        <v>27486</v>
       </c>
     </row>
     <row r="498" spans="1:10">
@@ -18663,7 +18663,7 @@
         <v>29.8</v>
       </c>
       <c r="J503">
-        <v>27661</v>
+        <v>125019</v>
       </c>
     </row>
     <row r="504" spans="1:10">
@@ -18823,7 +18823,7 @@
         <v>26.4</v>
       </c>
       <c r="J508">
-        <v>17577</v>
+        <v>50174</v>
       </c>
     </row>
     <row r="509" spans="1:10">
@@ -19111,7 +19111,7 @@
         <v>24.3</v>
       </c>
       <c r="J517">
-        <v>3122</v>
+        <v>15680</v>
       </c>
     </row>
     <row r="518" spans="1:10">
@@ -19559,7 +19559,7 @@
         <v>27.6</v>
       </c>
       <c r="J531">
-        <v>46741</v>
+        <v>35251</v>
       </c>
     </row>
     <row r="532" spans="1:10">
@@ -20263,7 +20263,7 @@
         <v>30.1</v>
       </c>
       <c r="J553">
-        <v>51152</v>
+        <v>206734</v>
       </c>
     </row>
     <row r="554" spans="1:10">
@@ -20519,7 +20519,7 @@
         <v>28</v>
       </c>
       <c r="J561">
-        <v>70176</v>
+        <v>149238</v>
       </c>
     </row>
     <row r="562" spans="1:10">
@@ -20551,7 +20551,7 @@
         <v>28.9</v>
       </c>
       <c r="J562">
-        <v>46580</v>
+        <v>318705</v>
       </c>
     </row>
     <row r="563" spans="1:10">
@@ -21127,7 +21127,7 @@
         <v>23.9</v>
       </c>
       <c r="J580">
-        <v>79422</v>
+        <v>121686</v>
       </c>
     </row>
     <row r="581" spans="1:10">
@@ -21703,7 +21703,7 @@
         <v>21.5</v>
       </c>
       <c r="J598">
-        <v>926694</v>
+        <v>30290</v>
       </c>
     </row>
     <row r="599" spans="1:10">
@@ -21831,7 +21831,7 @@
         <v>17.1</v>
       </c>
       <c r="J602">
-        <v>45864</v>
+        <v>26276</v>
       </c>
     </row>
     <row r="603" spans="1:10">
@@ -22023,7 +22023,7 @@
         <v>29.7</v>
       </c>
       <c r="J608">
-        <v>82097</v>
+        <v>56523</v>
       </c>
     </row>
     <row r="609" spans="1:10">
@@ -22119,7 +22119,7 @@
         <v>26.5</v>
       </c>
       <c r="J611">
-        <v>256358</v>
+        <v>156722</v>
       </c>
     </row>
     <row r="612" spans="1:10">
@@ -22535,7 +22535,7 @@
         <v>29.7</v>
       </c>
       <c r="J624">
-        <v>243714</v>
+        <v>134294</v>
       </c>
     </row>
     <row r="625" spans="1:10">
@@ -22631,7 +22631,7 @@
         <v>26.6</v>
       </c>
       <c r="J627">
-        <v>9630</v>
+        <v>39743</v>
       </c>
     </row>
     <row r="628" spans="1:10">
@@ -23047,7 +23047,7 @@
         <v>27.2</v>
       </c>
       <c r="J640">
-        <v>640428</v>
+        <v>344152</v>
       </c>
     </row>
     <row r="641" spans="1:10">
@@ -23687,7 +23687,7 @@
         <v>27</v>
       </c>
       <c r="J660">
-        <v>232859</v>
+        <v>369319</v>
       </c>
     </row>
     <row r="661" spans="1:10">
@@ -23815,7 +23815,7 @@
         <v>29.3</v>
       </c>
       <c r="J664">
-        <v>181768</v>
+        <v>172142</v>
       </c>
     </row>
     <row r="665" spans="1:10">
@@ -24487,7 +24487,7 @@
         <v>26.7</v>
       </c>
       <c r="J685">
-        <v>143453</v>
+        <v>362844</v>
       </c>
     </row>
     <row r="686" spans="1:10">
@@ -24615,7 +24615,7 @@
         <v>21.3</v>
       </c>
       <c r="J689">
-        <v>465555</v>
+        <v>75296</v>
       </c>
     </row>
     <row r="690" spans="1:10">

</xml_diff>